<commit_message>
Polish event template: Instructions tab, Table A/B dropdowns, weight total
</commit_message>
<xml_diff>
--- a/TasteOff-Template.xlsx
+++ b/TasteOff-Template.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criteria" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Judges" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teams" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criteria" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Judges" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teams" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,7 +31,25 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00B5361F"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00E08A2C"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00E08A2C"/>
     </font>
   </fonts>
   <fills count="3">
@@ -58,9 +77,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,70 +451,118 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Event ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Event Name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Start Time</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Interval</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Admin Passcode</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Results Passcode</t>
+          <t>Taste Off — Event Setup</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>houbbq-2026</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>HouBBQ Throwdown 2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="A2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Fill in the four tabs below, then load this file into the app:</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Set up event  →  Upload a .xlsx/.csv file   (or share this as a Google Sheet and paste the link).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TABS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>• Event    — one row: the event name, serving start time, minutes between dishes, and optional passcodes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>• Criteria — one row per judging category. Weights are percentages and must add up to 100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>• Judges   — one row per judge. Table must be A or B (each judge only sees their table's dishes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>• Teams    — one row per dish/restaurant. Code is the BLIND number judges see (never the name).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             Dish # sets the serving order; Serve Time can be left blank to auto-fill from the schedule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             Dish Description shows on the judge's ballot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>• Judges never see team names — only the Code. Names are revealed on the results screen after judging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>• You can add/remove rows freely. Leave a cell blank to omit it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>• The example below is the HouBBQ Throwdown 2026 event — overwrite it with your own.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -502,192 +575,70 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Criterion</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Short</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Weight %</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>High</t>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Event ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Event Name</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Start Time</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Interval</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Admin Passcode</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Results Passcode</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Use of Ingredients</t>
+          <t>houbbq-2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ingredients</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>30</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Basic / Uninspired</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Clever / Creative Use</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Flavor</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Flavor</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>25</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Bland / One-note</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Rich, Flavorful and Varied</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Dish Execution</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Execution</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>15</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Sloppy</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Composed and Amazing</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Appearance</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Appearance</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>12</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Visually Unappealing</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Stunning</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Creativity</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Creativity</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>10</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Could come from anywhere</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>One of a Kind!</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Texture</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Texture</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>8</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Tough / Chewy</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Tender and Amazing</t>
-        </is>
-      </c>
+          <t>HouBBQ Throwdown 2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -700,83 +651,202 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Judge</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Table</t>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Criterion</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Weight %</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Buckman</t>
+          <t>Use of Ingredients</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Ingredients</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Basic / Uninspired</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Clever / Creative Use</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Mueller</t>
+          <t>Flavor</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Flavor</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>25</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Bland / One-note</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Rich, Flavorful and Varied</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ong</t>
+          <t>Dish Execution</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Execution</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sloppy</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Composed and Amazing</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Timmonsw</t>
+          <t>Appearance</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Appearance</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Visually Unappealing</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Stunning</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kelly</t>
+          <t>Creativity</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
+          <t>Creativity</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Could come from anywhere</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>One of a Kind!</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Texture</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Texture</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Tough / Chewy</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Tender and Amazing</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL →</t>
+        </is>
+      </c>
+      <c r="C8" s="5">
+        <f>SUM(C2:C7)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -785,6 +855,101 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Judge</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Buckman</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mueller</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ong</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Timmonsw</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Kelly</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"A,B"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -798,36 +963,36 @@
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Team</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Table</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Dish #</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Serve Time</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Dish Description</t>
         </is>
@@ -1172,6 +1337,11 @@
       <c r="F14" t="inlineStr"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"A,B"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>